<commit_message>
update gerber file names
</commit_message>
<xml_diff>
--- a/hardware/devBoard/manufacture/devBoard BOM JLC.xlsx
+++ b/hardware/devBoard/manufacture/devBoard BOM JLC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\GitHub\Embedded-Systems-Instructor\Manufacturing Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\GitHub\Embedded-Systems-Instructor\hardware\devBoard\manufacture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A5197E-1E96-4F2B-BFCC-92875C678E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F3AB37-D88A-419E-961A-4F949FF4C626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -254,9 +254,6 @@
     <t>C131974</t>
   </si>
   <si>
-    <t>C132162</t>
-  </si>
-  <si>
     <t>C962159</t>
   </si>
   <si>
@@ -308,10 +305,13 @@
     <t>C883127</t>
   </si>
   <si>
-    <t>C25168846</t>
-  </si>
-  <si>
-    <t>C3039330</t>
+    <t>C69082</t>
+  </si>
+  <si>
+    <t>C5342990</t>
+  </si>
+  <si>
+    <t>C91144</t>
   </si>
 </sst>
 </file>
@@ -935,7 +935,7 @@
         <v>53</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -949,7 +949,7 @@
         <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -963,7 +963,7 @@
         <v>54</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -977,7 +977,7 @@
         <v>54</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -991,7 +991,7 @@
         <v>54</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1005,7 +1005,7 @@
         <v>54</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1019,7 +1019,7 @@
         <v>54</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1033,7 +1033,7 @@
         <v>54</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1047,7 +1047,7 @@
         <v>54</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -1062,7 +1062,7 @@
         <v>54</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1165,7 +1165,7 @@
         <v>63</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1179,7 +1179,7 @@
         <v>64</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1221,7 +1221,7 @@
         <v>1</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1235,7 +1235,7 @@
         <v>62</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1249,7 +1249,7 @@
         <v>66</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1263,7 +1263,7 @@
         <v>66</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1288,7 +1288,7 @@
         <v>65</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1302,7 +1302,7 @@
         <v>2</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>